<commit_message>
Update village feed (7h lookback)
</commit_message>
<xml_diff>
--- a/data/google_news_dedup_01_0426_UTC_past2d.xlsx
+++ b/data/google_news_dedup_01_0426_UTC_past2d.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DHL Supply Chain Expands Airport Role With Air France-KLM - Supply Chain Digital Magazine</t>
+          <t>Air France selects DHL Supply Chain to deliver ground handling services at London Gatwick - Parcel and Postal Technology International</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DHL Supply Chain Expands Airport Role With Air France-KLM - Supply Chain Digital Magazine</t>
+          <t>Air France selects DHL Supply Chain to deliver ground handling services at London Gatwick - Parcel and Postal Technology International</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 11:25:58 GMT</t>
+          <t>Wed, 01 Apr 2026 13:52:05 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPRTRERzh1akhtTExIWFAzVlhBandsTExpeTVqelZfOVNxa1pXRGFkdS1zVkZwQWNQd3dxRk5SSUlFaWdRWGdrYVpqSXEzTks2aFRtNTliSzBKMmhyOS1iMHZoeGhLYjAtS2F2dDhmMXBucDZrejF3N3Y2YjN0WEpoaQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNXzEwQ1A1dmZkeWRoVmJyTGE4NHFjb01mdU1Ud3ZTa1RyeG94Vmp5dndjTDlxTzE1emczUjZfZnZJbW5PRVk1X3laemRrRUJKcWl6Ty1mXzUzSUgtWDFTSnFaOVZYR1Jkb1B3dFdYazBwUm1ONi1TdWpMWHhMUEtNdXNyRzZudmkxNV91aEw1OWxuc0NZbEp3Y2hpVE5TelBjdkFyTjFQc0lrN0RTejIxc3hzLXJvbE1LdTdta0dtTlFwdXktSWxvTVc1VVVFcm5lR3dsdHlhdXgyQnBMcUExS200T084SDJjTHBkWXZ0dk5YWGtWX1VNMTJKMUZ6VjQ5d0R6WGN5NmlNUnM?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46113.47636574074</v>
+        <v>46113.57783564815</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Logistics Companies</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Dropit" OR "DHL" OR "UPS" OR "DPD" OR "Flight Logistics" OR "Fedex" OR "Amazon" OR "Royal Mail" OR "Parcelforce" OR "EVRI" ) AND ( "supply " OR  "delivery") AND -"postal vote"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Schietpartij Anderlecht: slachtoffer kreeg kogel in arm - Nieuwsblad</t>
+          <t>DHL Supply Chain Expands Airport Role With Air France-KLM - Supply Chain Digital Magazine</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Anderlecht shooting: victim was shot in the arm - Nieuwsblad</t>
+          <t>DHL Supply Chain Expands Airport Role With Air France-KLM - Supply Chain Digital Magazine</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 11:40:48 GMT</t>
+          <t>Wed, 01 Apr 2026 11:25:58 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPWHU0dllKMlNxUkJiVWI0M3RFMkxUZlpVZHhMcDVTal9rQzVua3BEQ2Y5NGtqbnRzSEhpTXdTUFUzTlZWQV9qQlFjUUotWkVHaDVvaV9DbjY0dEY5TG1HOHczZE5mZ3hoM3lVckJqUmFfXzM4dkVCWFF0Z2tQbkEyVkFvZVJpZjJyQ21ocVotYmFjc2FRbjdoZmpUa2xic2Z5UHd1YVhTcDh4QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPRTRERzh1akhtTExIWFAzVlhBandsTExpeTVqelZfOVNxa1pXRGFkdS1zVkZwQWNQd3dxRk5SSUlFaWdRWGdrYVpqSXEzTks2aFRtNTliSzBKMmhyOS1iMHZoeGhLYjAtS2F2dDhmMXBucDZrejF3N3Y2YjN0WEpoaQ?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,21 +570,21 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46113.48666666666</v>
+        <v>46113.47636574074</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>“Je gaat zien, je gaat branden”: Vrouwen veroordeeld voor explosie in Deurne - GVA</t>
+          <t>Man krijgt kogel in de arm bij schietpartij vlakbij metrostation Clemenceau in Anderlecht - VRT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>“You're going to see, you're going to burn”: Women convicted for explosion in Deurne - GVA</t>
+          <t>Man gets shot in the arm during shooting near Clemenceau metro station in Anderlecht - VRT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 10:47:41 GMT</t>
+          <t>Wed, 01 Apr 2026 14:42:24 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxQZmxiWlBGTjBrQnJtNnJMYUl1aW5adE9VaXlnOFViUkwwOWp6bHptS3FtQlVkMkVzTnR5YnZRbkQtOFRmbU9kXzZNV3psSUV0cjZNSk9aOVZEVGZzOXhMYzJDeUtXWGlabzBwQTFjajNQZVZJaG9wUHhHQXJ4WXk2VF9nRHB1OV9zUmJpTGtnakY4WU4wYzI1TXNQMjh3YVZRREZGU0lKa3FhMDMzQzdqN1lCRDJsdkdzazdxZEpVQS1VSTB1Y05TOXF2UW81TWRzR05rTWNDajVWZkR5N1lzeFhR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQVkRnNGhSV0NJN2lFZ2daX3RtY2stcU9ZbzlZaVhaT3NlcUliOU13NVowNFQzQkk3V1hYLWhfRzBBSmZBSUdlTzVDZzdoRng3aG1hUzRKdnVDbjNfbklqRlp3QjFWSU5XbnJrNXZ6dXM3cTdnNWFRRnZwaW8yQkRlRXNYZGp6UlJVY0QxQlU3NDM2aDRINVl3RDZMdFd5eEJTR3Q2OERMX1E?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46113.44978009259</v>
+        <v>46113.61277777778</v>
       </c>
     </row>
     <row r="5">
@@ -655,22 +655,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Jongen uit Friesland wilde aanslag plegen op Vlaams Parlement in Brussel - NRC</t>
+          <t>Schietpartij Anderlecht: slachtoffer kreeg kogel in arm - GVA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Boy from Friesland wanted to attack the Flemish Parliament in Brussels - NRC</t>
+          <t>Anderlecht shooting: victim was shot in the arm - GVA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 09:19:10 GMT</t>
+          <t>Wed, 01 Apr 2026 15:36:25 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQQzdqendJRW13bzNLejlNYk9zMU1oQ0d0c0ZGQy0zS3JsU25YN3dPcFhaQVk1Vl9pc3U3Zlg0aE9mYnRhNzI3Rm5ucnZGUHRobHNIaVR0aVFkb0ZubWRkNVFrVEQtOXBGU1ZVRnZkSWtnUklpZW94SjJrMkk0RThVbE50V0RIc3ZOOFBXVFQ5M1owa3lWSkl1d3RqUHB5aGg1b0I0YzRXcXUxdDJ2X1VscjFIdFZPQVpuYXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxNa0Fmc2VMRmNLWTMyZmlNXzVJYjVnUDFuenNnSmNWdEd6ZlZ5TlNKWW1SWk1pU0dXSTdyeHFHdXRQT2pCYzJlZDZXektWVFh2THp4TE8xZXduXzFmMHBhTE1pZ2hQYjFObnNRTU03eElrdjczNWpTcHcwRUp2QXRjUFFpTmJremFHSGt3V3BB?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46113.38831018518</v>
+        <v>46113.65028935186</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tiger Woods wil zich laten behandelen na arrestatie in Florida - HBVL</t>
+          <t>“Iemand die 1.500 euro wil verdienen?”: hoe een 13-jarige Nederlander een aanslag op het Vlaams Parlement plande - HLN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Tiger Woods wants treatment after arrest in Florida - HBVL</t>
+          <t>“Someone who wants to earn 1,500 euros?”: how a 13-year-old Dutchman planned an attack on the Flemish Parliament - HLN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 07:11:46 GMT</t>
+          <t>Wed, 01 Apr 2026 15:37:53 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPZDg5bXdnMndQTVY5RzByb1I4MkF6ZkRJdjRDOWpQdHVQSExveGZjNXZZMTVwWlE2Nm1mTDFRbF9rQjBCQ2k4UmQ4QmNUOC1YWV92bnRVTFMyRFFXMjM2aFpqVWJfOFlaN2IxSTFPRjBQNF9VNmZfNHhSVF82OXpoakl6Ri1CSXYyU01GaTJDLWhwWVBtQUZHUWVydlp1eVN5aUd0Sm1GcmpaWDVHTWFvaGxPYUtUZkowOUE4ckgybWE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOUW9WTG9iN3E4SWYzOUNTc1NxREIxSFlBSjM2RUlZTUlMZzdHa0RRTnZzTnJvbzJwclJmTVpwNWh4OFFjTUhrdUNhd3hIZjRidk10X0JEbzc1bTY4T25paTFPVXdOX2tGVTdZVlRoaFFicHBLZzE1ZmxXSUxHNlI5bTROX3BFSy1sUmhER19iT0pXMS12eXgxY1ZsYmhiRTFMX0xNNUEtTUdtM21icC1MTVk2aGkyZE1uaWo3ZXh0ajRDMVhUVldqMm1aNlVzQjdqMUh2SFgtSzE3NDVXck4xMU5R?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46113.29983796296</v>
+        <v>46113.65130787037</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ASSISEN. Zus van Davy Verachtert richt zich tot Cherkaoui: "Waar is uw schuldgevoel?" - GVA</t>
+          <t>“Je gaat zien, je gaat branden”: Vrouwen veroordeeld voor explosie in Deurne - Nieuwsblad</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ASSIS. Davy Verachtert's sister addresses Cherkaoui: "Where is your guilt?" - GVA</t>
+          <t>“You're going to see, you're going to burn”: Women convicted for explosion in Deurne - Nieuwsblad</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 12:59:46 GMT</t>
+          <t>Wed, 01 Apr 2026 10:45:46 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPN3JSYm1nanotcjdodlQwR2UyaTl4TjM5NlNhcXF4M0VFM05mNUlvenFTWkdScHl0OHdjeEhwc2F5eXcxS2s1bXBhTy10b2xuM1N3Q2hfLXp1aFNIbkxMWDAtNWRhZzZ3d3lhRWNNNW5DSUQ5NmIxeVk1WlRlaEwxVDNuZVloM0d6R1dLdEJxR3ZoUWJnZDZoU0xhVmtZWFhOb2ZTNXBfZkVEbkdNYU05bHEza3Z3Ulc3TFVQY2lKejQ4T2dDLTFLSUpsZERQNG9mZFVGaFZ5blhzQ0hNYjNzZGxmaGEzNmVsREt5c1VkOXFSXzUxdjY5dA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPdzNMYjZHUXNMdmhrYkI5LURrclVwZFZYdWRqcm4tc1k1R1lRWkdqX0p0M1d4T09uSnJ2S0M4bEF4YTVacldJQUkwVVFpVU4xMkIxZ3VLY24wOExHcVhSbUlyS1ZaTktRbThJWmtoTWlMSDFqQ0ZqX3JOMFVrN0Z6cW8yNnMxeE54dDUxSWlXejFsUGxVSE5RVWt0VTBKc1V2NDl1UGE2MDE1cTVRUFg3S1pZeWxwQ2FIXzRSS3hjeXlsVjZ5SmFCcUN1T3BJUG1HbWNfZnRRdHhFRHNPUVNpQmpTa2R5YTN2X253?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46113.54150462963</v>
+        <v>46113.44844907407</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Kennedytunnel volgende week twee nachten gesloten voor onderhoudswerken - Nieuwsblad</t>
+          <t>Staking bij De Lijn wegens schrappen van buslijn die de chauffeurs zélf nodig hebben: “Dit gaat ten koste van hun vrije tijd” - GVA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Kennedy tunnel closed for two nights next week for maintenance work - Nieuwsblad</t>
+          <t>Strike at De Lijn due to the cancellation of a bus line that the drivers themselves need: “This is at the expense of their free time” - GVA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 11:22:07 GMT</t>
+          <t>Wed, 01 Apr 2026 11:02:27 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxQWEx3d0FKT0ZIaWNjT1lLb0Ftb1FjRXEzaTlKTlBhcjMxOWtEYmRzdFEtYUFqV2p3WUlfMGNlT0pwS0Eydk9ONm1PeXhBSjJRZHF1bVAzMnlabGlfRFd2MEUxQVNuaS1aN2NOYlY4Rkdnc2FFZjE4alRRNTl6MVNSVmJ0YmM4SmVUamxjWV9SUmk5NWdQb1JOdEtHUTRscUpJc0ZBTGVxM0hqeUo4RFlRWnlfYWl0bVItOXMxVXEzS0h0Q3BjVllfanh1ejVPM2VJbVEtS05xRzV3Y01ZWkRNeDlOb2otRktqQnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxNajlMRHUzcTN2SlpadHBCOVd1ZTdMUkpfT2xMY0F6WEc3Y09Qek9FM2FSa3BNcHJ6cDVaQ3otTTBqUXFTVV9JVE85WjBkX004X09fTndPZnVWVmE0ZWNlckF1SG1VOFozRUZJazBMQktaaGtPSDhXX3NGeGF5LXVBT2ZDbHZzcWVoSDNRbzV5bTFGaHRfZlVkSllDcFZxRUgzaUhSYVBLSXRJbFFKQUVPWW95dUVTTFVvMUZWTTZNMEppZ0cyVmg3dkpNVGxRQnNHU1JSbGdoblRHTjZjRFIxdnotbHB5T0JhMi1wSU84TUY4N2lET1ZSa3NyUmllMUQ0dFJCcGFYR1Y0TXY2dWc?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,38 +859,38 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46113.47369212963</v>
+        <v>46113.46003472222</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dutch minor convicted over plans to attack Flemish Parliament - belganewsagency.eu</t>
+          <t>Morgen opnieuw bussen in regio Antwerpen nadat buschauffeurs spontaan werk neerlegden aan stelplaats in Mortsel - VRT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Dutch minor convicted over plans to attack Flemish Parliament - belganewsagency.eu</t>
+          <t>Buses again in the Antwerp region tomorrow after bus drivers spontaneously stopped work at the depot in Mortsel - VRT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 06:51:00 GMT</t>
+          <t>Wed, 01 Apr 2026 16:26:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNdzM0OXVKZXctRVdYS1F0UGZQeUxQVVE1eVplNW5LZ2xBU1doRUNaUjJxb000SUc2ekVmYnNoLVNHSXM0TWZsZ01odzN6aE9pMmp6bnJlWnlWMVBhQlZaM3VsMTBLRlRNNmYyVXFOcHN0eHhXeFNCQTVPeVJuUGttQkZnbmFHTWtiRmVTTWVGd1dEdWkyZjZZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNeHBXZU9TeTJBUTRVSzFaOVhiYjFrSUg4OGk0cEFLMjMzTUJXclU2a2JRY081VlZlLXFUTjZUcHNscE9EbXpVbm56VWhPVmJONnhGekE0ekNuVzZ4UUd4dFZtckFZaHdXcnVSMVNnUy1aS0lDMlo4R3E3Tlc5Wmd2a1hR?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46113.28541666667</v>
+        <v>46113.68472222222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Brussels introduces nighttime closures to combat crime around North Station - belganewsagency.eu</t>
+          <t>ASSISEN. Zus van Davy Verachtert richt zich tot Cherkaoui: "Waar is uw schuldgevoel?" - GVA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Brussels introduces nighttime closures to combat crime around North Station - belganewsagency.eu</t>
+          <t>ASSIS. Davy Verachtert's sister addresses Cherkaoui: "Where is your guilt?" - GVA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 11:01:00 GMT</t>
+          <t>Wed, 01 Apr 2026 12:59:46 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNaENpdWdTS2UxTmRFeDF2b2ZXOHM4Rk5Tc042TTVVbU96SlVTRkc4VGticTNlX0M3blJsUTUyUk9IY1FQQU9HU3NRRUJVTDRGd0J5SVltMXg0WGhZM0FjTHJ6WFdzMWRnVlg0OFltenJkbklzWmVScjFfTWpaNGVsV2pncXlBNlhCdzRSRXN5ZFByTWxNZ1h1WncxeDVWQXk0RkZ6YkdJOWNQZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxPN3JSYm1nanotcjdodlQwR2UyaTl4TjM5NlNhcXF4M0VFM05mNUlvenFTWkdScHl0OHdjeEhwc2F5eXcxS2s1bXBhTy10b2xuM1N3Q2hfLXp1aFNIbkxMWDAtNWRhZzZ3d3lhRWNNNW5DSUQ5NmIxeVk1WlRlaEwxVDNuZVloM0d6R1dLdEJxR3ZoUWJnZDZoU0xhVmtZWFhOb2ZTNXBfZkVEbkdNYU05bHEza3Z3Ulc3TFVQY2lKejQ4T2dDLTFLSUpsZERQNG9mZFVGaFZ5blhzQ0hNYjNzZGxmaGEzNmVsREt5c1VkOXFSXzUxdjY5dA?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46113.45902777778</v>
+        <v>46113.54150462963</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Watch 9News Latest Stories - Season 2026 - Savannah Guthrie's first interview since the disappearance of her mother - 9Now</t>
+          <t>Kennedytunnel volgende week twee nachten gesloten voor onderhoudswerken - Nieuwsblad</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Watch 9News Latest Stories - Season 2026 - Savannah Guthrie's first interview since the disappearance of her mother - 9Now</t>
+          <t>Kennedy tunnel closed for two nights next week for maintenance work - Nieuwsblad</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 07:19:54 GMT</t>
+          <t>Wed, 01 Apr 2026 11:22:07 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNV3RTc25YbGd0WXJYV29WOHpiNTZwckJwQi1OM0oySXNFZUFMMzdwQXFXX2hzUWZqSGdfNTBUb1JoV0Y1N19tQkVKaTNjS0dsdFdWbWZMSkxxWjE0bWxnTlRNT1NOTExzMm11RFpuakJ5eXQtdURkTl9NckJUS1ZQellBTDVTUkpJNWc2eA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxQWEx3d0FKT0ZIaWNjT1lLb0Ftb1FjRXEzaTlKTlBhcjMxOWtEYmRzdFEtYUFqV2p3WUlfMGNlT0pwS0Eydk9ONm1PeXhBSjJRZHF1bVAzMnlabGlfRFd2MEUxQVNuaS1aN2NOYlY4Rkdnc2FFZjE4alRRNTl6MVNSVmJ0YmM4SmVUamxjWV9SUmk5NWdQb1JOdEtHUTRscUpJc0ZBTGVxM0hqeUo4RFlRWnlfYWl0bVItOXMxVXEzS0h0Q3BjVllfanh1ejVPM2VJbVEtS05xRzV3Y01ZWkRNeDlOb2otRktqQnc?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46113.30548611111</v>
+        <v>46113.47369212963</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Watch 9News Latest Stories - Season 2026 - Tributes flow for beloved TV personality Mel Schilling - 9Now</t>
+          <t>Minderjarige jongen veroor­deeld voor voorbereiden extreemrechtse aanslagen in Nederland en België - de Volkskrant</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Watch 9News Latest Stories - Season 2026 - Tributes flow for beloved TV personality Mel Schilling - 9Now</t>
+          <t>Underage boy convicted of preparing far-right attacks in the Netherlands and Belgium - de Volkskrant</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 06:47:21 GMT</t>
+          <t>Wed, 01 Apr 2026 12:03:59 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOTWVFVVpTU1BxVXlTV0VrNHJzdVpuUEFISkpGaEs5RzlwZGR0LUJzQ2V0MWxuc2xpd1UtOVRJbERGWXYtblVxNGFKVEVWdnF3N29sazJhd00xWXgwWk5iVy1sSGpTNE92aHk5di1vOVNIMlBKU1VmZWE2cDBnSUdMTE5qVkxBV1BNN3c2Tw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQcVRVTU5mSjBXdWZNbG1WdG5ZU21hdDVTOEp6NWhqN2FXOEM4aXNkdjdNMktZVEIyYXFIRUgxYXRQX2Q1MXNOTlkwRzB0MWZWRHgxbXFBV2JEanV5eTVkc0NvVElvbUVIaFI3OEoxTWNWc2k5blAtcUpXOFFRM1EwX1RlZFNSdGI3MWJiWHUyQlI0ZnBJNmI1TWhOeTRHbTFiZW1LdTN3YThnb0hhX29uWDFWXzV2SHhHdEpNd3BySUZmbUwzeWhFbXJNbHdjQnl5SVd3RThrYTF0V19TREE?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46113.28288194445</v>
+        <v>46113.5027662037</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Un enfant de 12 ans planifiait un attentat contre le parlement flamand à Bruxelles - parismatch.be</t>
+          <t>Dutch schoolboy convicted of planning terror attack on Flemish Parliament in Brussels - The Brussels Times</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>A 12-year-old child planned an attack against the Flemish parliament in Brussels - parismatch.be</t>
+          <t>Dutch schoolboy convicted of planning terror attack on Flemish Parliament in Brussels - The Brussels Times</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 06:54:00 GMT</t>
+          <t>Wed, 01 Apr 2026 12:56:24 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxPcjczODJtRUppVC1LLTh1UlBJeU9UNlpIZ3lTajVvWURHaTh5RlAwSHp6Zm5zYUprZ2lUblp0bi1JN0g3R2lHQmlGSV9YU3pRV3RKOTJFcXpGU1dYMjlLTzVKYlg0aGhHX2I4MUlmeG5mSm1wdkZEMDh1VDl0NENlYW1RUzFtcFluTFVVVXc1TmZJdUZPZl93RUhyMGJMMU1CdjhxRlVnZC02d3l6Nk5ielV0Tk5BcU8yMmFCV0FGdEFfM1FJVllOM2pMY1RYSVV2TGZZeXIzdFhUeGctOFRoV25hUmwyWm1RcVRmd3lHT25weXVIVUtz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOUHlqcW05c211WjZyMW9UXzlIcVBMa24waTY5VldsQU9xNjJBdFRfcTcyeVRBMlB2aS1rUy1wN0RJMkJGTDBlcEhyVmlmdXBacXVaZjhHTEk2OVFNbnI1WEcxbHlDTG1na3F5Z2JZNFIyQ0c2OVZ1bkZFQVktU1RZRWhsR2NEXzZxNHhIRTM1aWlXMlRaanFmYkRCaHVtZktCQ2xiay1OUXFUSVY5bVptM1REcjNTRWFMaThQYV80NjJzXzhWaG5LcVVPaw?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46113.2875</v>
+        <v>46113.53916666667</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Un tout jeune adolescent condamné aux Pays-Bas pour avoir planifié un attentat contre le Parlement flamand - VRT</t>
+          <t>Brussels introduces nighttime closures to combat crime around North Station - belganewsagency.eu</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>A very young teenager sentenced in the Netherlands for planning an attack against the Flemish Parliament - VRT</t>
+          <t>Brussels introduces nighttime closures to combat crime around North Station - belganewsagency.eu</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 08:39:30 GMT</t>
+          <t>Wed, 01 Apr 2026 11:01:00 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQVHN0a2ZiYmhVSV9ieDBvWXVGdFZVZ2lueE5Bc2pFSnI3V1BGOGdEb0tsYWFVWlZYNXVKU2lfN3pEOEN1aE1uRmpzMFpjTm1hOTh2TW8zcDNXNTBCVm5GN29sbTFVcHhzXzRQUVZlaGxzV1VvbnN3NzRwSUVuMWx3S3BmY3NlaGxxbDdoaGF2RTZUZy1JOHBJMFR1eE0zQ1VGdng5OHB5Qm0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNaENpdWdTS2UxTmRFeDF2b2ZXOHM4Rk5Tc042TTVVbU96SlVTRkc4VGticTNlX0M3blJsUTUyUk9IY1FQQU9HU3NRRUJVTDRGd0J5SVltMXg0WGhZM0FjTHJ6WFdzMWRnVlg0OFltenJkbklzWmVScjFfTWpaNGVsV2pncXlBNlhCdzRSRXN5ZFByTWxNZ1h1WncxeDVWQXk0RkZ6YkdJOWNQZw?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,11 +1185,11 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46113.36076388889</v>
+        <v>46113.45902777778</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Konjufca : L'attentat de Banjska, le dernier clou dans le cercueil du dialogue de Bruxelles - koha.net</t>
+          <t>Nouvelle fusillade à Anderlecht: une personne blessée par balle - 7sur7.be</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Konjufca: The Banjska attack, the final nail in the coffin of the Brussels dialogue - koha.net</t>
+          <t>New shooting in Anderlecht: one person injured by gunfire - 7sur7.be</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 09:32:51 GMT</t>
+          <t>Wed, 01 Apr 2026 14:16:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOUENOTWNVY3U5RzA5OE1ZUWhCbkFpTUtha1ZUeWdWVmVreHc5TFhKZEFraWU5bXQ5Vm1HbzdjMUw2X0tMM3JyS2hWTjVLN1pfdWQ0NzU5WmtEczMwcngzamJCMDIwZDlrY2xhUHVhUE8ydjlEVWx0c2ZOUkFoSExNSTBRMXdnbXdCd2xQdTZFbW9TOG4zM3hvbkRPcWs0RmtIb213RHd0ZkkxZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPNTNVdDE3UnJoLVR4YnZsazhaRjdMRE9fenY4Z05YU0tEVS0xcU9uOGQ2aFhXdG5xX2tvZnBMN2RSb2dveWh0TWFmVEpXQmU5eE8xMmY0SkxjNEViMHhrbWxrSWxJRV8yUXQ0NEJxNEtic3lvMXhKRVVQUmJpdE9pd3lJRVl3MXJWQWJpdExMVXpuRkVuUHh5STRmODJMMjFCT3ZidTEtOGs4SXc?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46113.3978125</v>
+        <v>46113.59444444445</v>
       </c>
     </row>
     <row r="16">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Un million de cigarettes contrefaites saisies à Bruxelles - BruxellesToday</t>
+          <t>Immigration: quand Trump inspire les européens sur les expulsions de migrants - lanouvelletribune.info</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>One million counterfeit cigarettes seized in Brussels - BruxellesToday</t>
+          <t>Immigration: when Trump inspires Europeans on expulsions of migrants - lanouvelletribune.info</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 07:11:21 GMT</t>
+          <t>Wed, 01 Apr 2026 14:22:26 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPcG1JMTFsWGxveHdsVkNubW9mRndWT0ZUXzlZdDkwOVVVbTRrZDd3Zi12S1JlU1J3blJpV0JZeGFYYUtySl9sVG01MmZweklKdjB3MXdRaHY5UVphM25RcmhfS1hxVDRFUkNJTlRhSTFPWlNUTktqRDdfUjJZTk5GQVBwNGd2RDlMaGVRREV1YkhlU2p6UGxHOGpsNlU5MkJTSUJN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNNm04bThRcktoTWwxOF9VcjNHMjc2WmFlWnJIaThILWM1dXk1OUc2cDFjMURaVDhuVmsySEdRMHptQWZ5SUZ2R1ZTZUdrSDMxVjBNbnV5TlhlQm1OOWNQcWRWTG5pMDJHMV9YRThmNGphdWtVVFdoRlJsSFhTajVFTVF4d01xWUllaFFSWWI3MS1CZ18tQm5xQUo3RnVPM1NaeGs4a3dkc25CTElmWWlKMDdmMTdpWjA?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46113.29954861111</v>
+        <v>46113.59891203704</v>
       </c>
     </row>
     <row r="19">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Drie mannen opgepakt na gewelddadige overval op vrouw in Blankenberge: verdachten blijken niet aan hun proefstuk toe - VRT</t>
+          <t>Drie jaar cel voor vrouw uit Beringen die collega belaagde na onbeantwoorde liefde: "Stond zelfs naakt op de oprit" - VRT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Three men arrested after violent robbery of woman in Blankenberge: suspects appear not to be up to their test - VRT</t>
+          <t>Three years in prison for woman from Beringen who attacked colleague after unrequited love: "Even stood naked in the driveway" - VRT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 13:12:24 GMT</t>
+          <t>Wed, 01 Apr 2026 14:27:50 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNU0FYWElHS1lIRDFhYnk5RlRxa3czZno1X29LSjNOVG5xRnZ3ZXp4MUtrODNGdHdiMWlja1R2ODNoTFR3TjFNdkwwWU1ycnFWaElBc1ljRUdGcWhHcUxyRnRucGxDTWc4R256Ymo4cEJYSEVCQWZfMkppU1VBQUZ5WjItWmxQTTU4RVRRdzZUZmUxQ3VtVzB5QkpwSG1CckRzMkdRSTZmTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQNkFSOEh2YkdxcnhoUmpzcUZFeXp0NmZvelhyMnpKOWNiM0Nta2VBdU1uZHExSmZZRFVuVmpyV0JJYTlTQmlROUI1STduVmFQemRheHlZMGFEM0Z3aDdGYXVZelZVTDNDV2hWTTF1QS1hNk5VQWRaYWl1UUhZaGFJaUduWFNyZw?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,38 +1464,38 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46113.55027777778</v>
+        <v>46113.60266203704</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Contours flous de la photographie wallonne - La Libre.be</t>
+          <t>Injures discriminatoires et cyberharcèlement aggravé : Booba sèche une nouvelle fois son procès - Libération</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Blurred contours of Walloon photography - La Libre.be</t>
+          <t>Discriminatory insults and aggravated cyberharassment: Booba once again skips his trial - Libération</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 08:18:00 GMT</t>
+          <t>Wed, 01 Apr 2026 14:15:00 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNaUo1VnZlNWtTVFE5V2Vkc2FHNEVlYjJicEhlZEt3a1J0X2tlT0JGVVZwRHc1VUtubm02SnhIZmdOZ0FQcE1yMTdCcDc0Wmdsa0t2WEpQc28wRkJuMEYwM2ptY2VtekVGZXZ2WENpQlFOZFRsZUJUWF9sTWlxTXJPRkhlME1rUjhJQ0dKbUZzRkhjLVJpczJRYzdnMS1QY1p1TWJqMzFDcEJ0cDk2M3hpaEx5OEh4WTNu?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNQ3k0bVJJalhUV3NoVzdLUnh6MlZLdjdLdkRHcnFmSExJNk5qMEF3YmZWT3k1TmZJUzJqQlVaNkppSDVYR0UyX29sY1RKQ2tMYnNuemFkWTFFRldiMmlIb1N3OWxXTTZ0UkhJeUxVekdMYkUzY19OMkNudDNtanhZZzA1eXdfUDZiSUFFbWhGQWZ1SVNzSHc0Sk90LWtrZ3JhWEtrejFMU2tPaDdIaXMtSzY0cFNLaENwWTFrZUY2eGNOVE1BYXFsVndHN0lFUU8wajdQUm9NWGZfNm5XV0ZlRlNJYXh0alVzZ3l2MjNWV0JnbjY1dHp3aGRoTEcwNVhvOWFvd2RmUEQwSDA?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1519,13 +1519,13 @@
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46113.34583333333</v>
+        <v>46113.59375</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Découvrez ici les 8 tendances mode pour le printemps/été 2026 - ELLE.be</t>
+          <t>France's Dassault says 'weeks' left to save Europe warplane project - France 24</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Discover here the 8 fashion trends for spring/summer 2026 - ELLE.be</t>
+          <t>France's Dassault says 'weeks' left to save Europe warplane project - France 24</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 13:08:42 GMT</t>
+          <t>Wed, 01 Apr 2026 10:41:12 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOVld5Y2dlbC1FSlJodGNjR2ljalVZZEdFZ0FPQ3lkN1B6OVFzQm9vVXNuR2EzOTBZMlFDZnk3d0Rzb1ZVTXRyS2ZOUlBuYUpPWEpGNzdPLUFPdUVIdjRsVm1NUTBVMWVibDhVY1l4dHM1ZDhSbTNWTVYzdXJmOUdENkg1RWd2RkZreEVFRmZRYUZHTFFnMWVSYg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQMFJzWmdhYTJvU0xXdnhqcDIyS05RcFdfTlZrbTJuN244c0JjZkFVb0RzY0xUMDBteS16NFlNcXVwWGhhdVBmaDVzTlJhWFRNMnpnUXJLbFhESjh6Vlc0d2xwMUtkS2tQZjlGd3V3MzRGQmdDbVhBV3lLOGtmaG9KcUYxdjhXOEY5LVNHSWU5X3VHVjdad2U3RDRwak1QMGljUUU5NG16azJ5NTlDSEVwWDlB?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46113.54770833333</v>
+        <v>46113.44527777778</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>La CGT bloque un hypermarché Auchan à Bagnolet - information.tv5monde.com</t>
+          <t>Zimmer brennt: Polizei ermittelt - augsburger-allgemeine.de</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>The CGT blocks an Auchan hypermarket in Bagnolet - information.tv5monde.com</t>
+          <t>Room is on fire: police investigate - augsburger- Allgemeine.de</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 11:46:07 GMT</t>
+          <t>Wed, 01 Apr 2026 12:13:32 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQakMwRXY5Yll0amVqMFlQcER5RGhwUG01VmhicnRwRmhObWtueTlSMmZianZTbDhia25oamtqWDVpaHpQRVlVTkVNQmJ1dG1zYVZhY3UtMXNMMUtkNmhzRlVoLWwzMGxBTGdULXlSMWVDZGVhMHZzamI1V2RUNGtaYWppNDVYXzNEXzZid3ViNjJiRHpQX3RDcFhR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQMm5YYUc0SDF0VExNVUx0SVlneTZnZWQ1bHNKdkZjRkNKYy1jYXNNUVVKeVJZa2FzR1pmUUU4M1phWFJpdXRKUmlrTVA0bFYtRjc1dkFZRmd6M25zRmd4VDZtMXVIU2tKQlU5UEMxYVN2Ry1rMHBHblFiQm1sWEZ5ekZpWXhLUjZRcXplMzVzRlNBLVNiU0g3cnFEUmZ6Zw?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46113.4903587963</v>
+        <v>46113.50939814815</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Meurtre de Quentin : Raphaël Arnault sort enfin du silence et se pose en victime - lejdd.fr</t>
+          <t>FC Ingolstadt 04 vs. FC Erzgebirge Aue - Live Score - May 03, 2026 - FOX Sports</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Murder of Quentin: Raphaël Arnault finally comes out of silence and poses as a victim - lejdd.fr</t>
+          <t>FC Ingolstadt 04 vs. FC Erzgebirge Aue - Live Score - May 03, 2026 - FOX Sports</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 08:48:56 GMT</t>
+          <t>Wed, 01 Apr 2026 12:07:23 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNd3pKUUpIb0F6TmttZzV1Wjg3aHBJalRjWENjVmNyM2s5d1E0MkEzd1NhR1BqOVFBS1RtcTJrMWpPVi1kcm5OSlo2TlRTN1MwM0ZVZVQ0Z0d5M3ltV0ZjWkZGYWRhUmtuQnplUmtaRXVyY2lNbnFRbmlIQUNJTEhLNUx0cmc2cldaYTdFeFFxdlZEenlLbEcyUDRrbzU0WXhMa2JEcVdkd2ZPR0stb1JsdDViWGhLZ2s?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNWWJzNnFLRlpUbkZmaE56UzVZMVZaeU11dUVEVXpVMEhhNlNROURrT3NqNkVIMDNqaTdpTWtMNkRKNzVMd19vWElxMkdJc3I3Vm42WEhEWE0zNzA4azNZcTRSV0Y5c1ZET0tkMVJsWktkSXJNdVc1ZC1PTEd3aXgtRjBfTW4wMnNkUml0ZXRVUXVXUHRZbVI4ZWZXLUxwRThSNUF0OUZ3?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46113.36731481482</v>
+        <v>46113.50512731481</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>France's Dassault says 'weeks' left to save Europe warplane project - France 24</t>
+          <t>Woman in her 80s stabbed to death outside home in Shooters Hill - london-now.co.uk</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>France's Dassault says 'weeks' left to save Europe warplane project - France 24</t>
+          <t>Woman in her 80s stabbed to death outside home in Shooters Hill - london-now.co.uk</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 10:41:12 GMT</t>
+          <t>Wed, 01 Apr 2026 15:23:01 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQMFJzWmdhYTJvU0xXdnhqcDIyS05RcFdfTlZrbTJuN244c0JjZkFVb0RzY0xUMDBteS16NFlNcXVwWGhhdVBmaDVzTlJhWFRNMnpnUXJLbFhESjh6Vlc0d2xwMUtkS2tQZjlGd3V3MzRGQmdDbVhBV3lLOGtmaG9KcUYxdjhXOEY5LVNHSWU5X3VHVjdad2U3RDRwak1QMGljUUU5NG16azJ5NTlDSEVwWDlB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQclNYelFnS1FXLS02bmJhbFRwaE93cXFMdTZiNmJOQTYxeWY4NHdNdVFoNHY3SE9PRi12eFJsVzRFUk5laWh4QnNDMVp6RUctcXI0V2lqcFR2aXRkdUNjMUwyQlVtUEhyNHJJMUlsdm85WENqWktfS1VtcF9qaDJwdlNlRG5uRnNlYkRFbV9weFdzTzdNMmNNOVVn?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1739,38 +1739,38 @@
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46113.44527777778</v>
+        <v>46113.64098379629</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Zimmer brennt: Polizei ermittelt - Augsburger Allgemeine</t>
+          <t>Armed police rush to shooting with ‘bullet casings scattered on the floor’ - london-now.co.uk</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Room is on fire: Police investigate - Augsburger Allgemeine</t>
+          <t>Armed police rush to shooting with ‘bullet casings scattered on the floor’ - london-now.co.uk</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 12:13:32 GMT</t>
+          <t>Wed, 01 Apr 2026 15:51:11 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQMm5YYUc0SDF0VExNVUx0SVlneTZnZWQ1bHNKdkZjRkNKYy1jYXNNUVVKeVJZa2FzR1pmUUU4M1phWFJpdXRKUmlrTVA0bFYtRjc1dkFZRmd6M25zRmd4VDZtMXVIU2tKQlU5UEMxYVN2Ry1rMHBHblFiQm1sWEZ5ekZpWXhLUjZRcXplMzVzRlNBLVNiU0g3cnFEUmZ6Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQRElBdFFaaGdQT25DbHhlaC1jY3Z6Y2FQcDJGLTZjbGFOYmpBRlEtTl8zYURkd2tXanp6dC1rOWJxRjdJWWZYbWlHN0k4MHB1UHMwVHktajktOHNKTC1aUHZhMEZVX2pKMFRwRTJrM2YwV1ZtU1Rmdks4aXF6LU1ZT1hadExQYmZNR3l0Q0U4SDlBQ3RJclZOdHlOSkg?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46113.50939814815</v>
+        <v>46113.66054398148</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>High Level City UK Ireland</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FC Ingolstadt 04 vs. FC Erzgebirge Aue - Live Score - May 03, 2026 - foxsports.com</t>
+          <t>Woman (63) charged with murder after Dublin house party stabbing ‘too unwell’ to attend hearing - Sunday World</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>FC Ingolstadt 04 vs. FC Erzgebirge Aue - Live Score - May 03, 2026 - foxsports.com</t>
+          <t>Woman (63) charged with murder after Dublin house party stabbing ‘too unwell’ to attend hearing - Sunday World</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 12:07:23 GMT</t>
+          <t>Wed, 01 Apr 2026 16:19:59 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNWWJzNnFLRlpUbkZmaE56UzVZMVZaeU11dUVEVXpVMEhhNlNROURrT3NqNkVIMDNqaTdpTWtMNkRKNzVMd19vWElxMkdJc3I3Vm42WEhEWE0zNzA4azNZcTRSV0Y5c1ZET0tkMVJsWktkSXJNdVc1ZC1PTEd3aXgtRjBfTW4wMnNkUml0ZXRVUXVXUHRZbVI4ZWZXLUxwRThSNUF0OUZ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQOEU2dEVBcnVUbTVTMkRkR0pDeElOYzRIek1nM2dqRWpRd0FEeDJXaVZFci1LbVZndG1IUDJfcTlVelN6a2FfYXRKVy1RaWt0S1pLV3NvQ0RuTy01eUE0UDlQYmJzV0hJSHVBOWtsRnVydkxHTmF2eDZNVFBRdWl5V1JMTHROWExCVFZKVXkzNXV1azVNVWdfalpRM0VjWnd3d1RiRDBaWkZZUGQ4cVV3dVdEWDFhbjVQTTJoOGNrY3V4dVQ3YVI3X2NRT0xtNEVpR0NhM0ZvWXBKUQ?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46113.50512731481</v>
+        <v>46113.68054398148</v>
       </c>
     </row>
     <row r="27">
@@ -1865,22 +1865,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026 film and high-end TV productions shooting in the UK and Ireland: latest updates - Screen Daily</t>
+          <t>Lurgan proxy bomb attempt ‘would have caused devastation’, Long says - london-now.co.uk</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026 film and high-end TV productions shooting in the UK and Ireland: latest updates - Screen Daily</t>
+          <t>Lurgan proxy bomb attempt ‘would have caused devastation’, Long says - london-now.co.uk</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 07:29:48 GMT</t>
+          <t>Wed, 01 Apr 2026 14:25:54 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQZmNMRTBhWHdsbFo0WHUtenBKUWJ0Z09LVVBuTjVUb1R6dnYyV0UwSEluX01NUXJuVzhuVlZCTUlHanpOQ0hpT1p4N2xGSnIyaEg3eGRKQ3BZVlJWT0hPREU4dmd2azc2VGVhQVl2emFKVmpENnNrT3BJNGVDY2xlNDVSUV95dzdPcHFtOHhqcG9WbUdYYU9odjhUTHp2b0dzMTZ6Yzh4U1VGNVVfeVl5RmQ1eDJpLU91MHlMUS1kZlZNNng3LTE1VHNIb1o?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPWi1ISUJ5SC1vLWltdWlDWm1IOEdBcUdtRVF2S0s2VkZHN09Yc21Wd3g0N250NjRtZVVybjk5TWJuSlE0cThtVXZZalR6amRNYXprZGRTYm1tTUl3RWZIQ210WmdfVXVxbTZtelpfaEhMc2VSaVhLQ2lXbWxNd29SRUxNSmtMU2VvdVJTNGJ5LWxQTkoxbXhKNlJZUkI4VE1GUDZLQkxMZ3ZQeEJPX2xGRkZ4RQ?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1904,38 +1904,38 @@
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46113.31236111111</v>
+        <v>46113.60131944445</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Murder hunt after man, 29, shot dead sitting in car outside Euston Station - London Evening Standard</t>
+          <t>La Pavoni, la protesta dei lavoratori a Milano - Il Cittadino di Lodi</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Murder hunt after man, 29, shot dead sitting in car outside Euston Station - London Evening Standard</t>
+          <t>La Pavoni, the workers' protest in Milan - Il Cittadino di Lodi</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 10:38:08 GMT</t>
+          <t>Wed, 01 Apr 2026 14:28:53 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQRTB1OGl4VjZ5ZFlkenNneFRSTzZSRnRRQWxrQzAzVWlndWIwTUMzcmxLQk1fUS1YYUlISU52YzNVNG5PZzRtcU9uUVhKY245RnNQZzMtekRzLVl2VFNrLWVILUlJRnhIQ3JfckwyX21nNVFpVmRybDUteUwyR1lTMm9GQmFVYnBhX0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQeWsweDFNMGNfWkFOdTlnejFlZVNrNnMwaG1ZUUtXMkN5RzMxUmZ4ZHVaV3FnRjBjRGdmRFVYOXRGUmN1OFhHRUt5REsyUmZLb3pNZlVJUzJoeWR2YVpIWTI5ejZxVEpUZW5zMlpGLXpxVmRWMlgyQVF3SnNySk9YQVNRX1Fxal9UUDBqMkhfb1NVRkpsQUpiSmtWM3JZOWhuSUE?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46113.44314814815</v>
+        <v>46113.6033912037</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>High Level City UK Ireland</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Dublin" OR "Oxford" OR "London") AND ("Bomb" OR "explosion" OR "shooting"  OR "Stabbing" OR "suspicious package" OR "unattended Package" OR "explosive" OR "bomb threat" )</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Man, 18, charged with murder after stabbing near Westminster Abbey - London Now</t>
+          <t>Leoncavallo, il Viminale non molla sul risarcimento. Associazione Mamme: “Contro di noi una causa infondata e politica” - Il Giorno</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Man, 18, charged with murder after stabbing near Westminster Abbey - London Now</t>
+          <t>Leoncavallo, the Interior Ministry does not give up on compensation. Mothers Association: “An unfounded and political lawsuit against us” - Il Giorno</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 07:47:40 GMT</t>
+          <t>Wed, 01 Apr 2026 11:48:54 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNTS1lVHJYV0k1ZldkZmM3dk5qU0xyd2dfQTNra3dYMmM4N2t1UllndFJRc0FiaTZVbUluZG1uQTEtQnV1Q255bzgxNkkxdXNjaE9WVTlSaGJudnRVTTJndGNEb1ZoOWV1bEFQU0pmN0xTWGZUQUIxNUUyZFhlN3hmbkF6elVnRXVvMEdvZVZ1OXlzeFZ2dGFCTEdJd0ctcWtp?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPbkM4VWZmdF9WNVppMXlNd21nRkJCSzdYc3drYXJmZ0FWMVJKa3c1QklBQk5VVlRzOVUzLXlsaDhhVFJRcEhFUmtGVG5XM0NHVWtLWDRlYWFFbEtCeUJWQXNIYndCaGItdGhzamY1Z25OZGE5S3I1aW9JLUdid0dOMEhYSV9JNGVrcGlsRk9vbzVQSDU5T212c3ZwTXg1cUJhdlE?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46113.32476851852</v>
+        <v>46113.49229166667</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>High Level City France French</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Paris" OR "Île-de-France") AND ("alerte à la bombe" OR "colis suspect" OR "menace à la bombe" OR fusillade OR "attentat" OR "attaque au couteau" OR "opération de police" OR évacuation) AND -immobilier AND -"prix immobilier" AND -foot AND -transfert AND -Texas</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Attentat déjoué contre la Bank of America à Paris : une information judiciaire ouverte pour association de malfaiteurs terroriste - Le Monde.fr</t>
+          <t>Lombardia. Opposizioni, sindacati e cittadini promuovono manifestazione per il diritto alla salute - Quotidiano Sanità</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Attack foiled against the Bank of America in Paris: judicial investigation opened for terrorist conspiracy - Le Monde.fr</t>
+          <t>Lombardy. Oppositions, unions and citizens promote demonstration for the right to health - Quotidiano Sanità</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 09:28:14 GMT</t>
+          <t>Wed, 01 Apr 2026 12:39:00 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAJBVV95cUxQOEotTDVqUFF6ampQSTZ0a3BSMVVPeGRhd1czSU0tc01ROG5JRmRKTExLQk5BcEtPNF9UT2RsRERXQUNzdWpvbzl4ZFE3VlhnRG8zYWN3bDBJbUNma040NnZHa1hwMVQ4RThUdlA5TGFPVHJ2RVhUUTF4c0JzYXNLbEtCZVc3ZHlJSVd4SUFtTm96T1E0NVhXUmxzd1lGbjFidmpzT25uVDhBVTljNVlJeUhJV2FfbUN1ZWx1V2RzeG9ib0JEUWJfbkJ2cnZJMk9iQU1uTWo5WVRDVndFN1d5c29yb19NYmRHSV9faGlFbFl2SlIxX0NUSnhyZ2p6WkNEYUtFd1ExaGhMZm1Ub2hKSTlsUlRfdlY4N2luWDZuZlA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNZngxRWMzLXkzTFhMZWdRcTIycTFLZUlmMTRRNGlHWExyc3IzM08tdFg4LU83bHgxN1ZQZThkWVV2U0FhLTV0MlhlemlocTdwRXh4SGZwOGxQVms5Rzd2aWtISVhwUHFWak1kcm9OUWZ3ZEh5RHdIOUlaTzJmOHBjNXRPUDNHRGRTWGo4RWNOcTRTRk9XOHNvYUN6S0hKMG5NbXJMVXVRNW5DWXlTdVhzemloYVd3ZmcwR0pMdnpOM3dIVGxVaWdIc2NneGppT1NjVVNjRVd3?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,21 +2055,21 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>FR:fr</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46113.39460648148</v>
+        <v>46113.52708333333</v>
       </c>
     </row>
     <row r="31">
@@ -2085,22 +2085,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Leoncavallo, il Viminale non molla sul risarcimento. Associazione Mamme: “Contro di noi una causa infondata e politica” - ilgiorno.it</t>
+          <t>Bloccata la linea Caserta-Foggia, caos treni a Bari: ritardi e corse cancellate - BariToday</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Leoncavallo, the Interior Ministry does not give up on compensation. Mothers Association: “An unfounded and political lawsuit against us” - ilgiorno.it</t>
+          <t>The Caserta-Foggia line blocked, train chaos in Bari: delays and canceled journeys - BariToday</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Wed, 01 Apr 2026 11:48:54 GMT</t>
+          <t>Wed, 01 Apr 2026 16:07:00 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPbkM4VWZmdF9WNVppMXlNd21nRkJCSzdYc3drYXJmZ0FWMVJKa3c1QklBQk5VVlRzOVUzLXlsaDhhVFJRcEhFUmtGVG5XM0NHVWtLWDRlYWFFbEtCeUJWQXNIYndCaGItdGhzamY1Z25OZGE5S3I1aW9JLUdid0dOMEhYSV9JNGVrcGlsRk9vbzVQSDU5T212c3ZwTXg1cUJhdlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxORzVmaWt0MmxDaHFFVGVQZzF1Ym12U1FCNUxZMWNkdHpVVXNOWmJBU1ExWEgtVTdIdENYVm5pYjJ2UzJueHJyNUVxV2xOazBTYmNVQ2Zib3ZIWEtuSktTQUowQ2UwOGh4RUFRZDJzVXd4QS1wcjlZbDJ5ZnpyVHFHdW9uVVdQTzdPaXpXeDU2dTM?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2124,62 +2124,7 @@
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46113.49229166667</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Perché Nordio ha deciso di mandare gli ispettori presso il tribunale di Bologna - BolognaToday</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Why Nordio decided to send inspectors to the Bologna court - BolognaToday</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Wed, 01 Apr 2026 07:37:50 GMT</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPMmh2TFd5NkN3M3ZTVDQyMXZaeWVlYVgzMDBjeEstYkdubGg2dFNwNGNfV2xMR0RZcXdWQkR1WnZ1MUg5M2dCOXp3SUltc0t4NklwY0g3UEMxaE1aaUlTMXRvMnVPaWhCYUNqZTdHYmlJcm85LUVoVVQybERQNUdubjRNal95aHlqZE5DQTM3aEJ1QXJ6aXU4?oc=5</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K32" s="1" t="n">
-        <v>46113.31793981481</v>
+        <v>46113.67152777778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>